<commit_message>
update ai log, IEEE
</commit_message>
<xml_diff>
--- a/ai_logs/Nguyên_AILog.xlsx
+++ b/ai_logs/Nguyên_AILog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\SUM26\CSD\CSD201-group3\ai_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB3022D-5A4B-4EE5-8CC3-3B42851A5B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BE6E8C-8F3F-48C1-A103-7DF9D3A896C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -1010,33 +1010,33 @@
     <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1359,11 +1359,11 @@
       <c r="A1" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1621,25 +1621,25 @@
       <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -1772,7 +1772,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="238.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="37" t="s">
         <v>194</v>
       </c>
       <c r="B8" s="20" t="s">
@@ -1798,7 +1798,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="301.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="38" t="s">
         <v>195</v>
       </c>
       <c r="B9" s="25" t="s">
@@ -1824,7 +1824,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="233.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="38" t="s">
         <v>196</v>
       </c>
       <c r="B10" s="28" t="s">
@@ -1850,7 +1850,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="276.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="38" t="s">
         <v>197</v>
       </c>
       <c r="B11" s="20" t="s">
@@ -2036,24 +2036,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -2116,7 +2116,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="148.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="39" t="s">
         <v>194</v>
       </c>
       <c r="B6" s="35" t="s">
@@ -2136,7 +2136,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="123" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="39" t="s">
         <v>195</v>
       </c>
       <c r="B7" s="35" t="s">
@@ -2384,17 +2384,17 @@
       <c r="A1" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">

</xml_diff>

<commit_message>
update AI Log and files data
</commit_message>
<xml_diff>
--- a/ai_logs/Nguyên_AILog.xlsx
+++ b/ai_logs/Nguyên_AILog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\SUM26\CSD\CSD201-group3\ai_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BE6E8C-8F3F-48C1-A103-7DF9D3A896C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA2146B-FB9A-47CF-8F13-2A0DBB056CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="267">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -76,9 +76,6 @@
   </si>
   <si>
     <t>Nhóm cần chọn 1 topic từ đề RQ_CSD201_CSD203 và xác định cấu trúc dữ liệu lõi cho hệ thống Browser History &amp; Cache Navigation (Topic 9)</t>
-  </si>
-  <si>
-    <t>"theo m thì topic nào dễ nhất" (kèm RQ_CSD201_CSD203.docx) → "phân tích bài toán và cho biết những yêu cầu bắt buộc của project, sau đó tiến hành lập kế hoạch thực hiện"</t>
   </si>
   <si>
     <t>AI gợi ý Topic 9 (Browser History) dễ nhất trong danh sách đề tài. Đề xuất 2 lựa chọn cấu trúc dữ liệu: Doubly Linked List (di chuyển tiến/lùi dễ dàng) hoặc Stack (lưu để back về trang trước). Lập kế hoạch Tuần 1 gồm Decomposition (chia Node, BrowserHistory, methods) và Abstraction (so sánh DLL vs Stack theo bối cảnh thực tế).</t>
@@ -664,6 +661,589 @@
   </si>
   <si>
     <t>Thêm footnote vào slide RQ2: 'Benchmark includes JIT warmup; actual amortized time may vary. For production-grade measurement, JMH is recommended.'; giữ câu chốt AI cho phần trả lời GV nhưng bổ sung khi bị hỏi sâu.</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>Nhiều flowchart được lưu thành các file riêng khiến báo cáo khó theo dõi và trình bày. Cần quyết định cách tổng hợp để thuận tiện cho GitHub và báo cáo.</t>
+  </si>
+  <si>
+    <t>"trong thư mục diagram, có nhiều flowchart nằm riêng biệt vs nhau, hãy gộp chung các ảnh flowchart vào 1 file để dễ trình bày hơn, không gộp thành 1 ảnh nhé"</t>
+  </si>
+  <si>
+    <t>Sau khi tạo Markdown, cần định dạng tài liệu vừa hiển thị ảnh vừa có thể bổ sung phần mô tả chi tiết cho từng flowchart.</t>
+  </si>
+  <si>
+    <t>AI đề xuất chuyển sang file HTML, hiển thị đầy đủ các flowchart và thêm vùng văn bản dưới mỗi hình để người dùng bổ sung giải thích.</t>
+  </si>
+  <si>
+    <t>Cần xác nhận khi push lên GitHub thì các flowchart trong Markdown có hiển thị trực tiếp hay chỉ hiện dưới dạng liên kết.</t>
+  </si>
+  <si>
+    <t>"nếu như hiển thị trên github thì nó sẽ hiện ra ảnh hay link dẫn đến ảnh"</t>
+  </si>
+  <si>
+    <t>Nhóm cần lựa chọn nền tảng và template phù hợp để viết báo cáo IEEE cho dự án Browser History.</t>
+  </si>
+  <si>
+    <t>"hướng dẫn viết IEEE bằng latex cho dự án Browser History này"</t>
+  </si>
+  <si>
+    <t>AI đề xuất sử dụng Overleaf cùng template IEEE Conference và xây dựng khung bài báo gồm Abstract, Introduction, Architecture, Implementation, Performance Evaluation và Conclusion.</t>
+  </si>
+  <si>
+    <t>Khung IEEE ban đầu còn ngắn và chưa phản ánh đầy đủ các module Browser History.</t>
+  </si>
+  <si>
+    <t>AI mở rộng toàn bộ bài báo bằng tiếng Anh, bổ sung phần System Architecture, Implementation Details, Benchmark, Complexity Analysis và Future Work.</t>
+  </si>
+  <si>
+    <t>Sau khi hoàn thành báo cáo IEEE, nhóm cần chuẩn bị kịch bản thuyết trình phù hợp với nội dung báo cáo và code.</t>
+  </si>
+  <si>
+    <t>AI đề xuất chia bài thuyết trình theo 4 phần: Giới thiệu, Lựa chọn cấu trúc dữ liệu, Demo hệ thống, Đánh giá hiệu năng và Benchmark.</t>
+  </si>
+  <si>
+    <t>Slide IEEE + Script thuyết trình + Demo Browser History.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: HTML linh hoạt hơn Markdown nhưng không hiển thị trực tiếp trên GitHub như README. Contextualization: Mục tiêu chính lúc này là phục vụ trình bày trực tiếp nên HTML phù hợp hơn. Creative Synthesis: Sử dụng HTML trong giai đoạn chỉnh sửa nội dung, sau đó chuyển lại Markdown để lưu trữ trên GitHub. Decision: Chấp nhận HTML như tài liệu tạm thời phục vụ chỉnh sửa.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI cung cấp khung chuẩn IEEE nhưng nội dung vẫn còn mang tính mẫu, cần điều chỉnh theo đúng dự án Browser History của nhóm. Contextualization: Môn CSD yêu cầu báo cáo theo chuẩn học thuật, việc dùng template IEEE giúp tiết kiệm thời gian định dạng. Creative Synthesis: Chọn Overleaf để nhiều thành viên cùng chỉnh sửa đồng thời, sau đó thay thế toàn bộ nội dung mẫu bằng nội dung thực tế của project. Decision: Áp dụng IEEE Conference Template làm chuẩn báo cáo chính thức.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Nội dung dài và học thuật hơn nhưng vẫn cần rà soát để đảm bảo khớp hoàn toàn với source code thực tế. Contextualization: Báo cáo sẽ được đối chiếu trực tiếp với code trong buổi bảo vệ. Creative Synthesis: Giữ lại cấu trúc và cách diễn đạt học thuật của AI, đồng thời chỉnh sửa các mô tả về hàm và độ phức tạp theo implementation cuối cùng của nhóm. Decision: Dùng bản mở rộng của AI làm nền cho báo cáo chính thức.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Kịch bản hợp lý nhưng cần cân đối thời lượng giữa các thành viên và tránh để một người trình bày quá nhiều nội dung kỹ thuật. Contextualization: Hội đồng đánh giá cả kiến thức thuật toán lẫn khả năng giải thích implementation. Creative Synthesis: Điều chỉnh kịch bản để mỗi thành viên trình bày một phần gắn với module mình phụ trách, kết hợp demo trực tiếp và biểu đồ benchmark. Decision: Áp dụng kịch bản AI làm khung, sau đó phân chia thời lượng đều cho từng thành viên.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI khẳng định Browser History sử dụng </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HashMap + Doubly Linked List</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và đạt O(1) cho mọi thao tác.</t>
+    </r>
+  </si>
+  <si>
+    <t>Unsupported assumption</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">So sánh với source code </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BrowserHistory.java</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Project Browser History thực tế chỉ sử dụng </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Doubly Linked List</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, chưa tích hợp HashMap. Chỉ project LRU Cache mới dùng HashMap + DLL.</t>
+    </r>
+  </si>
+  <si>
+    <t>Luôn đối chiếu mô tả thuật toán với implementation thực tế trước khi đưa vào báo cáo hoặc slide.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI mô tả Browser History có các module </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>DataGenerator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ExperimentRunner</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mặc định trong project.</t>
+    </r>
+  </si>
+  <si>
+    <t>Fabricated project structure</t>
+  </si>
+  <si>
+    <t>Kiểm tra cấu trúc project và repository.</t>
+  </si>
+  <si>
+    <t>Chỉ giữ các module thực sự tồn tại; nếu chưa có thì tự xây dựng hoặc loại bỏ khỏi báo cáo.</t>
+  </si>
+  <si>
+    <t>Không sử dụng nội dung AI sinh ra nếu chưa tồn tại trong project.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI cho rằng thao tác </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>truncateForward()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> luôn có độ phức tạp O(1).</t>
+    </r>
+  </si>
+  <si>
+    <t>Over-generalization</t>
+  </si>
+  <si>
+    <t>Phân tích source code và thuật toán.</t>
+  </si>
+  <si>
+    <t>Nếu hàm chỉ cập nhật pointer thì O(1); nếu còn duyệt hoặc giải phóng node thì cần phân tích lại. Báo cáo chỉ ghi theo implementation thực tế.</t>
+  </si>
+  <si>
+    <t>Độ phức tạp phải được xác minh từ code chứ không chỉ dựa trên mô tả lý thuyết.</t>
+  </si>
+  <si>
+    <t>AI khẳng định benchmark 100,000 requests chứng minh chắc chắn thuật toán đạt O(1).</t>
+  </si>
+  <si>
+    <t>Overclaim</t>
+  </si>
+  <si>
+    <t>So sánh giữa benchmark và phân tích Big-O.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Benchmark chỉ cho thấy thời gian gần như ổn định trong điều kiện thử nghiệm, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>không phải bằng chứng toán học</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của Big-O.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Phân biệt giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>empirical performance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>theoretical complexity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> trong báo cáo khoa học.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI tự thêm các hàm như </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>searchByTitle()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>removePage()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>loadFromCSV()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> vào phần IEEE.</t>
+    </r>
+  </si>
+  <si>
+    <t>Fabricated implementation</t>
+  </si>
+  <si>
+    <t>Đối chiếu với source code hiện tại.</t>
+  </si>
+  <si>
+    <t>Xóa hoặc sửa các mô tả không tồn tại trong project.</t>
+  </si>
+  <si>
+    <t>AI thường mở rộng nội dung để bài viết "đẹp" hơn, nhưng cần loại bỏ những chức năng chưa được implement.</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>0112</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>"dựa trên báo cáo của dự án, hướng dẫn trình bày bản IEEE này"</t>
+  </si>
+  <si>
+    <t>"chọn topic nào phù hợp với năng lực của nhóm" (kèm RQ_CSD201_CSD203.docx) → "phân tích bài toán và cho biết những yêu cầu bắt buộc của project, sau đó tiến hành lập kế hoạch thực hiện"</t>
+  </si>
+  <si>
+    <t>"tạo lại file tổng hợp dự án cho phần flowchart"</t>
+  </si>
+  <si>
+    <t>"viết bằng tiếng anh, bao gồm tất cả các phần nội dung đã được đề cập là sẽ báo cáo cho giảng viên"</t>
+  </si>
+  <si>
+    <r>
+      <t>all_flowcharts.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> chứa toàn bộ flowchart bằng Markdown.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>flowcharts_presentation.html</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> được tạo thành công.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>main.tex</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> phiên bản mở rộng trên Overleaf.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>AI đề xuất tạo một file Markdown (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>all_flowcharts.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) nhúng toàn bộ hình flowchart theo từng mục bằng đường dẫn tương đối thay vì ghép các ảnh thành một hình duy nhất.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Critical Thinking: Markdown giúp giữ nguyên chất lượng ảnh và dễ cập nhật từng flowchart riêng, nhưng chưa đáp ứng nhu cầu vừa ghi chú vừa trình bày như tài liệu. Contextualization: Repository GitHub cần tài liệu dễ đọc và có thể xem trực tiếp trên web. Creative Synthesis: Chấp nhận phương án Markdown để phục vụ GitHub, đồng thời cân nhắc định dạng khác (HTML/Word) cho việc thuyết trình. Decision: Sử dụng </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>all_flowcharts.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> làm tài liệu chính trong repository.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI giải thích cú pháp </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>![]()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> trong Markdown sẽ render trực tiếp hình ảnh nếu dùng đúng đường dẫn tương đối.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Critical Thinking: Không chỉ tin vào giải thích của AI mà cần đối chiếu với chuẩn Markdown của GitHub. Contextualization: Repository của môn học sẽ được giảng viên xem trực tiếp trên GitHub nên khả năng hiển thị ảnh là yêu cầu quan trọng. Creative Synthesis: Kiểm tra lại cấu trúc thư mục để đảm bảo toàn bộ đường dẫn ảnh đều là relative path (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>./image.png</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>). Decision: Giữ nguyên Markdown và sử dụng đường dẫn tương đối cho tất cả hình ảnh.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Preview GitHub hiển thị đầy đủ các flowchart trong </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>all_flowcharts.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Project Overleaf + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>main.tex</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -673,7 +1253,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -762,12 +1342,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -786,8 +1360,89 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -849,12 +1504,60 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -904,19 +1607,107 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -959,75 +1750,18 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1036,6 +1770,143 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1346,7 +2217,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -1355,225 +2226,225 @@
     <col min="5" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+    </row>
+    <row r="3" spans="1:6" ht="18" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-    </row>
-    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C4" t="s">
         <v>43</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="C5" t="s">
         <v>45</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="9" spans="1:6" ht="18" customHeight="1">
+      <c r="A9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="C10">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C10">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="C11" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C11" s="3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="C12" s="4">
         <f>C11/C10</f>
-        <v>0.15384615384615385</v>
+        <v>0.11666666666666667</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="C13" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="18" customHeight="1">
       <c r="A15" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="6" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="B16" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="6" t="s">
+    </row>
+    <row r="17" spans="1:5" ht="28.8">
+      <c r="A17" s="7" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="B17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.8">
+      <c r="A18" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C19" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28.8">
+      <c r="A21" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
+      <c r="D21" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18" customHeight="1">
+      <c r="A22" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="C21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="6" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
+      <c r="B23" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="6" t="s">
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="8">
+        <v>6</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="8">
-        <v>2</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5">
       <c r="A25" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" s="7" t="s">
         <v>12</v>
       </c>
@@ -1581,18 +2452,18 @@
         <v>2</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B27" s="8">
         <v>2</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1606,7 +2477,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -1617,326 +2488,431 @@
     <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-    </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1">
+      <c r="A2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-    </row>
-    <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+    </row>
+    <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1">
+      <c r="A3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="54" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="166.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:8" ht="166.2" customHeight="1">
+      <c r="A4" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="F4" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="G4" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="H4" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="22" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="165.6" customHeight="1">
+      <c r="A5" s="35" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="165.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="B5" s="36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="D5" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="38" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="220.8" customHeight="1">
+      <c r="A6" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="40" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="237" customHeight="1">
+      <c r="A7" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="238.2" customHeight="1">
+      <c r="A8" s="42" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="220.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="C8" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8" s="37" t="s">
+        <v>175</v>
+      </c>
+      <c r="G8" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="H8" s="37" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="301.8" customHeight="1">
+      <c r="A9" s="42" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="C9" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="H9" s="38" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="233.4" customHeight="1">
+      <c r="A10" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="237" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
+      <c r="D10" s="40" t="s">
+        <v>183</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="F10" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>186</v>
+      </c>
+      <c r="H10" s="40" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="276.60000000000002" customHeight="1">
+      <c r="A11" s="43" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="F11" s="37" t="s">
+        <v>190</v>
+      </c>
+      <c r="G11" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="29" customFormat="1" ht="195.6" customHeight="1">
+      <c r="A12" s="73">
+        <v>9</v>
+      </c>
+      <c r="B12" s="74" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="56" t="s">
+        <v>206</v>
+      </c>
+      <c r="E12" s="57" t="s">
+        <v>207</v>
+      </c>
+      <c r="F12" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="G12" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="H12" s="58" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="30" customFormat="1" ht="167.4" customHeight="1">
+      <c r="A13" s="75">
+        <v>10</v>
+      </c>
+      <c r="B13" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" s="22" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="238.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
-        <v>194</v>
-      </c>
-      <c r="B8" s="20" t="s">
+      <c r="C13" s="60" t="s">
+        <v>205</v>
+      </c>
+      <c r="D13" s="60" t="s">
+        <v>208</v>
+      </c>
+      <c r="E13" s="61" t="s">
+        <v>256</v>
+      </c>
+      <c r="F13" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="G13" s="60" t="s">
+        <v>220</v>
+      </c>
+      <c r="H13" s="62" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="31" customFormat="1" ht="168.6" customHeight="1">
+      <c r="A14" s="76">
         <v>11</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>174</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="F8" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>177</v>
-      </c>
-      <c r="H8" s="22" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="301.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="38" t="s">
-        <v>195</v>
-      </c>
-      <c r="B9" s="25" t="s">
+      <c r="B14" s="63" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="64" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="65" t="s">
+        <v>211</v>
+      </c>
+      <c r="F14" s="64" t="s">
+        <v>263</v>
+      </c>
+      <c r="G14" s="64" t="s">
+        <v>264</v>
+      </c>
+      <c r="H14" s="64" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="32" customFormat="1" ht="200.4" customHeight="1">
+      <c r="A15" s="76">
+        <v>12</v>
+      </c>
+      <c r="B15" s="76" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>180</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="G9" s="24" t="s">
-        <v>182</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="233.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="38" t="s">
-        <v>196</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>185</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>187</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="276.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="38" t="s">
-        <v>197</v>
-      </c>
-      <c r="B11" s="20" t="s">
+      <c r="D15" s="66" t="s">
+        <v>212</v>
+      </c>
+      <c r="E15" s="67" t="s">
+        <v>213</v>
+      </c>
+      <c r="F15" s="66" t="s">
+        <v>214</v>
+      </c>
+      <c r="G15" s="66" t="s">
+        <v>221</v>
+      </c>
+      <c r="H15" s="66" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="33" customFormat="1" ht="168.6" customHeight="1">
+      <c r="A16" s="76">
+        <v>13</v>
+      </c>
+      <c r="B16" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="D16" s="69" t="s">
+        <v>215</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>257</v>
+      </c>
+      <c r="F16" s="69" t="s">
+        <v>216</v>
+      </c>
+      <c r="G16" s="69" t="s">
+        <v>222</v>
+      </c>
+      <c r="H16" s="71" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="29" customFormat="1" ht="160.19999999999999" customHeight="1">
+      <c r="A17" s="76">
+        <v>14</v>
+      </c>
+      <c r="B17" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>189</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="G11" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="H11" s="22" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="124.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="56" t="s">
+        <v>217</v>
+      </c>
+      <c r="E17" s="57" t="s">
+        <v>254</v>
+      </c>
+      <c r="F17" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="G17" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="H17" s="56" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="79.95" customHeight="1">
+      <c r="A18" s="34"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+    </row>
+    <row r="19" spans="1:8" ht="79.95" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1946,7 +2922,7 @@
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
     </row>
-    <row r="20" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="79.95" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1956,7 +2932,7 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="79.95" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1966,7 +2942,7 @@
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
     </row>
-    <row r="22" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="79.95" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1976,7 +2952,7 @@
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
     </row>
-    <row r="23" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="79.95" customHeight="1">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1986,7 +2962,7 @@
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
     </row>
-    <row r="24" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="79.95" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1996,7 +2972,7 @@
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
     </row>
-    <row r="25" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="79.95" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -2006,7 +2982,7 @@
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
     </row>
-    <row r="26" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="79.95" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -2028,174 +3004,234 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+    </row>
+    <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1">
+      <c r="A3" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-    </row>
-    <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="B3" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="94.95" customHeight="1">
+      <c r="A4" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="48" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="94.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="26" t="s">
+      <c r="C4" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="D4" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="E4" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="F4" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="34" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="94.95" customHeight="1">
+      <c r="A5" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="48" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="94.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="35" t="s">
+      <c r="C5" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="36" t="s">
+      <c r="D5" s="49" t="s">
         <v>89</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="E5" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="F5" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="F5" s="36" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="148.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="39" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="148.19999999999999" customHeight="1">
+      <c r="A6" s="50" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>197</v>
+      </c>
+      <c r="D6" s="49" t="s">
+        <v>198</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>199</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="123" customHeight="1">
+      <c r="A7" s="50" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>198</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>199</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>200</v>
-      </c>
-      <c r="F6" s="36" t="s">
+      <c r="B7" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="49" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="123" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
-        <v>195</v>
-      </c>
-      <c r="B7" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="36" t="s">
+      <c r="D7" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="E7" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="E7" s="36" t="s">
+      <c r="F7" s="49" t="s">
         <v>204</v>
       </c>
-      <c r="F7" s="36" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:6" ht="127.2" customHeight="1">
+      <c r="A8" s="45" t="s">
+        <v>249</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="111.6" customHeight="1">
+      <c r="A9" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>230</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>232</v>
+      </c>
+      <c r="F9" s="46" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="108" customHeight="1">
+      <c r="A10" s="45" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>235</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>234</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>236</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>237</v>
+      </c>
+      <c r="F10" s="46" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="94.2" customHeight="1">
+      <c r="A11" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>240</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>239</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>241</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>242</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="63.6" customHeight="1">
+      <c r="A12" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>247</v>
+      </c>
+      <c r="F12" s="46" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="60" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -2203,47 +3239,42 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="60" customHeight="1">
       <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="60" customHeight="1">
       <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="60" customHeight="1">
       <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
     </row>
-    <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="60" customHeight="1">
       <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
-    <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="60" customHeight="1">
       <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
     </row>
-    <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="60" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -2251,7 +3282,7 @@
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
     </row>
-    <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="60" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -2259,7 +3290,7 @@
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
     </row>
-    <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="60" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -2267,7 +3298,7 @@
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
     </row>
-    <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="60" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -2275,7 +3306,7 @@
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
     </row>
-    <row r="23" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="60" customHeight="1">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -2283,7 +3314,7 @@
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
     </row>
-    <row r="24" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="60" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -2291,75 +3322,75 @@
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
     </row>
-    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="18" customHeight="1">
       <c r="A30" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="10" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="s">
+      <c r="B31" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="C31" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="10" t="s">
+    </row>
+    <row r="32" spans="1:6" ht="28.8" customHeight="1">
+      <c r="A32" s="7" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7" t="s">
+      <c r="B32" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="C32" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="7" t="s">
+    </row>
+    <row r="33" spans="1:3" ht="28.8" customHeight="1">
+      <c r="A33" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="B33" s="7" t="s">
+      <c r="C33" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C33" s="7" t="s">
+    </row>
+    <row r="34" spans="1:3" ht="28.8" customHeight="1">
+      <c r="A34" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C34" s="7" t="s">
+    </row>
+    <row r="35" spans="1:3" ht="28.8" customHeight="1">
+      <c r="A35" s="7" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="7" t="s">
+      <c r="B35" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C35" s="7" t="s">
+    </row>
+    <row r="36" spans="1:3" ht="43.2" customHeight="1">
+      <c r="A36" s="7" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="C36" s="7" t="s">
         <v>108</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2374,299 +3405,299 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="4" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-    </row>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="6" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="B5" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="11" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="34.200000000000003">
+      <c r="A6" s="12" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="B6" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="C6" s="72" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="D6" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="32" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="34.200000000000003">
+      <c r="A7" s="12" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="B7" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D7" s="32" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="34.200000000000003">
+      <c r="A8" s="12" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="B8" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C8" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D8" s="32" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="34.200000000000003">
+      <c r="A9" s="12" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="B9" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="C9" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C9" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="32" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="34.200000000000003">
+      <c r="A10" s="12" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="B10" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D10" s="32" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="18" customHeight="1">
+      <c r="A12" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:4">
+      <c r="A13" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="11" t="s">
+    <row r="14" spans="1:4" ht="22.8">
+      <c r="A14" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="13" t="s">
+      <c r="C14" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D14" s="32" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="22.8">
+      <c r="A15" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="B15" s="13" t="s">
+      <c r="C15" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C15" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D15" s="32" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="22.8">
+      <c r="A16" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="B16" s="13" t="s">
+      <c r="C16" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="C16" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D16" s="32" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="22.8">
+      <c r="A17" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="B17" s="13" t="s">
+      <c r="C17" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="C17" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D17" s="32" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="22.8">
+      <c r="A18" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="13" t="s">
+      <c r="C18" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="C18" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="D18" s="32" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="15.6" customHeight="1">
+      <c r="A20" s="14" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+    <row r="21" spans="1:4">
+      <c r="A21" s="15" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
+    <row r="22" spans="1:4">
+      <c r="A22" s="15" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
+    <row r="25" spans="1:4" ht="18" customHeight="1">
+      <c r="A25" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:4">
+      <c r="A26" s="16" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="43.2" customHeight="1">
       <c r="A27" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="D27" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:4" ht="49.95" customHeight="1">
       <c r="A28" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="33" t="s">
+      <c r="B28" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C28" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="D28" s="21" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="49.95" customHeight="1">
+      <c r="A29" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="D28" s="32" t="s">
+      <c r="C29" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="33" t="s">
-        <v>155</v>
-      </c>
-      <c r="C29" s="33" t="s">
+    <row r="30" spans="1:4" ht="49.95" customHeight="1">
+      <c r="A30" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="C30" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="33" t="s">
-        <v>157</v>
-      </c>
-      <c r="C30" s="33" t="s">
+    <row r="31" spans="1:4" ht="49.95" customHeight="1">
+      <c r="A31" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="C31" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>167</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="33" t="s">
-        <v>159</v>
-      </c>
-      <c r="C31" s="33" t="s">
-        <v>160</v>
-      </c>
-      <c r="D31" s="32" t="s">
-        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>